<commit_message>
plan-frm: rebuild FRM-EIB04 template จากไฟล์ตัวอย่างล่าสุด + remap FRM_STYLE
ตัวอย่าง/FRM-EIB04 (TP).xlsx ถูกแก้ใหม่ (ตัวอย่างข้อมูล 8→10 แถว ทำให้แถวปิดตาราง/
ลายเซ็นขยับจาก 26/27/28 เป็น 30/31/32 + cellXfs ทั้งตารางเรียงลำดับใหม่เกือบทั้งหมด
แม้ assert cellXfs=178 จะยังผ่านโดยบังเอิญ) รัน build-frm-eib04-template.ps1 ใหม่
แล้ว remap FRM_STYLE ใน 15-plan-export.js ทั้งชุด (first/item/close/sig1/sig2) จาก
แถว 10/12/30/31/32 ของไฟล์จริง ตรวจ semantic ทีละ style (font/border/alignment)
ไม่ใช่เดา offset; อัปเดต tests/plan-export.test.html ให้ตรง id ใหม่ (ALLPASS) +
verify เพิ่มด้วย Excel COM เปิดไฟล์ export จริงไม่ฟ้องซ่อม + ตรวจตำแหน่งกล่อง
Month/Year/Group/Unit/Section เทียบเส้นใต้ในฟอร์ม ยังตรงตำแหน่งเดิม + SW v89

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/frm-eib04-template.xlsx
+++ b/assets/frm-eib04-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\8014\Desktop\calibration-system-main\ตัวอย่าง\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F33F982-8F4E-4DF8-9DF4-EB1AEC33A7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12E9A9A-2F12-4D85-8CF5-4D7E578948C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1048,6 +1048,174 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1058,15 +1226,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1093,77 +1252,68 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1174,12 +1324,6 @@
     <xf numFmtId="0" fontId="9" fillId="11" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1221,150 +1365,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -1500,16 +1500,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>24764</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>247650</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>114299</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1539,8 +1539,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="3514725" y="85725"/>
-          <a:ext cx="428625" cy="457200"/>
+          <a:off x="4010024" y="15240"/>
+          <a:ext cx="523875" cy="544830"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7155,15 +7155,15 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="19.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13" style="1" customWidth="1"/>
     <col min="4" max="4" width="6.88671875" style="1" customWidth="1"/>
     <col min="5" max="5" width="8.33203125" style="1" customWidth="1"/>
     <col min="6" max="14" width="2.109375" style="1" customWidth="1"/>
     <col min="15" max="17" width="2.5546875" style="1" customWidth="1"/>
     <col min="18" max="18" width="2.44140625" style="1" customWidth="1"/>
     <col min="19" max="36" width="2.5546875" style="1" customWidth="1"/>
-    <col min="37" max="37" width="9" style="1" customWidth="1"/>
+    <col min="37" max="37" width="8.109375" style="1" customWidth="1"/>
     <col min="38" max="38" width="7.44140625" style="1" customWidth="1"/>
     <col min="39" max="39" width="8.44140625" style="1" customWidth="1"/>
     <col min="40" max="43" width="9.44140625" style="1" customWidth="1"/>
@@ -7174,51 +7174,51 @@
       <c r="AO1" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="29.25" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="102"/>
-      <c r="S3" s="102"/>
-      <c r="T3" s="102"/>
-      <c r="U3" s="102"/>
-      <c r="V3" s="102"/>
-      <c r="W3" s="102"/>
-      <c r="X3" s="102"/>
-      <c r="Y3" s="102"/>
-      <c r="Z3" s="102"/>
-      <c r="AA3" s="102"/>
-      <c r="AB3" s="102"/>
-      <c r="AC3" s="102"/>
-      <c r="AD3" s="102"/>
-      <c r="AE3" s="102"/>
-      <c r="AF3" s="102"/>
-      <c r="AG3" s="102"/>
-      <c r="AH3" s="102"/>
-      <c r="AI3" s="102"/>
-      <c r="AJ3" s="102"/>
-      <c r="AK3" s="102"/>
-      <c r="AL3" s="102"/>
-      <c r="AM3" s="102"/>
-      <c r="AN3" s="102"/>
-      <c r="AO3" s="102"/>
-      <c r="AP3" s="102"/>
-      <c r="AQ3" s="102"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="103"/>
+      <c r="Q3" s="103"/>
+      <c r="R3" s="103"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="103"/>
+      <c r="X3" s="103"/>
+      <c r="Y3" s="103"/>
+      <c r="Z3" s="103"/>
+      <c r="AA3" s="103"/>
+      <c r="AB3" s="103"/>
+      <c r="AC3" s="103"/>
+      <c r="AD3" s="103"/>
+      <c r="AE3" s="103"/>
+      <c r="AF3" s="103"/>
+      <c r="AG3" s="103"/>
+      <c r="AH3" s="103"/>
+      <c r="AI3" s="103"/>
+      <c r="AJ3" s="103"/>
+      <c r="AK3" s="103"/>
+      <c r="AL3" s="103"/>
+      <c r="AM3" s="103"/>
+      <c r="AN3" s="103"/>
+      <c r="AO3" s="103"/>
+      <c r="AP3" s="103"/>
+      <c r="AQ3" s="103"/>
     </row>
     <row r="4" spans="1:44" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F4" s="2" t="s">
@@ -7265,221 +7265,221 @@
       </c>
     </row>
     <row r="7" spans="1:44" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="114" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="72" t="s">
+      <c r="B7" s="128" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="75" t="s">
+      <c r="C7" s="114" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="78" t="s">
+      <c r="D7" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="81" t="s">
+      <c r="E7" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="84" t="s">
+      <c r="F7" s="137" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="85"/>
-      <c r="H7" s="85"/>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
-      <c r="L7" s="85"/>
-      <c r="M7" s="85"/>
-      <c r="N7" s="85"/>
-      <c r="O7" s="85"/>
-      <c r="P7" s="85"/>
-      <c r="Q7" s="85"/>
-      <c r="R7" s="85"/>
-      <c r="S7" s="85"/>
-      <c r="T7" s="85"/>
-      <c r="U7" s="85"/>
-      <c r="V7" s="85"/>
-      <c r="W7" s="85"/>
-      <c r="X7" s="85"/>
-      <c r="Y7" s="85"/>
-      <c r="Z7" s="85"/>
-      <c r="AA7" s="85"/>
-      <c r="AB7" s="85"/>
-      <c r="AC7" s="85"/>
-      <c r="AD7" s="85"/>
-      <c r="AE7" s="85"/>
-      <c r="AF7" s="85"/>
-      <c r="AG7" s="85"/>
-      <c r="AH7" s="85"/>
-      <c r="AI7" s="85"/>
-      <c r="AJ7" s="86"/>
-      <c r="AK7" s="109" t="s">
+      <c r="G7" s="138"/>
+      <c r="H7" s="138"/>
+      <c r="I7" s="138"/>
+      <c r="J7" s="138"/>
+      <c r="K7" s="138"/>
+      <c r="L7" s="138"/>
+      <c r="M7" s="138"/>
+      <c r="N7" s="138"/>
+      <c r="O7" s="138"/>
+      <c r="P7" s="138"/>
+      <c r="Q7" s="138"/>
+      <c r="R7" s="138"/>
+      <c r="S7" s="138"/>
+      <c r="T7" s="138"/>
+      <c r="U7" s="138"/>
+      <c r="V7" s="138"/>
+      <c r="W7" s="138"/>
+      <c r="X7" s="138"/>
+      <c r="Y7" s="138"/>
+      <c r="Z7" s="138"/>
+      <c r="AA7" s="138"/>
+      <c r="AB7" s="138"/>
+      <c r="AC7" s="138"/>
+      <c r="AD7" s="138"/>
+      <c r="AE7" s="138"/>
+      <c r="AF7" s="138"/>
+      <c r="AG7" s="138"/>
+      <c r="AH7" s="138"/>
+      <c r="AI7" s="138"/>
+      <c r="AJ7" s="139"/>
+      <c r="AK7" s="112" t="s">
         <v>23</v>
       </c>
-      <c r="AL7" s="109"/>
-      <c r="AM7" s="109"/>
-      <c r="AN7" s="109"/>
-      <c r="AO7" s="109"/>
-      <c r="AP7" s="109"/>
-      <c r="AQ7" s="110"/>
+      <c r="AL7" s="112"/>
+      <c r="AM7" s="112"/>
+      <c r="AN7" s="112"/>
+      <c r="AO7" s="112"/>
+      <c r="AP7" s="112"/>
+      <c r="AQ7" s="113"/>
     </row>
     <row r="8" spans="1:44" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="76"/>
-      <c r="B8" s="73"/>
-      <c r="C8" s="76"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="98">
+      <c r="A8" s="115"/>
+      <c r="B8" s="129"/>
+      <c r="C8" s="115"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="135"/>
+      <c r="F8" s="126">
         <v>1</v>
       </c>
-      <c r="G8" s="87">
+      <c r="G8" s="104">
         <v>2</v>
       </c>
-      <c r="H8" s="87">
+      <c r="H8" s="104">
         <v>3</v>
       </c>
-      <c r="I8" s="87">
+      <c r="I8" s="104">
         <v>4</v>
       </c>
-      <c r="J8" s="87">
+      <c r="J8" s="104">
         <v>5</v>
       </c>
-      <c r="K8" s="87">
+      <c r="K8" s="104">
         <v>6</v>
       </c>
-      <c r="L8" s="87">
+      <c r="L8" s="104">
         <v>7</v>
       </c>
-      <c r="M8" s="87">
+      <c r="M8" s="104">
         <v>8</v>
       </c>
-      <c r="N8" s="87">
+      <c r="N8" s="104">
         <v>9</v>
       </c>
-      <c r="O8" s="87">
+      <c r="O8" s="104">
         <v>10</v>
       </c>
-      <c r="P8" s="87">
+      <c r="P8" s="104">
         <v>11</v>
       </c>
-      <c r="Q8" s="87">
+      <c r="Q8" s="104">
         <v>12</v>
       </c>
-      <c r="R8" s="87">
+      <c r="R8" s="104">
         <v>13</v>
       </c>
-      <c r="S8" s="87">
+      <c r="S8" s="104">
         <v>14</v>
       </c>
-      <c r="T8" s="87">
+      <c r="T8" s="104">
         <v>15</v>
       </c>
-      <c r="U8" s="87">
+      <c r="U8" s="104">
         <v>16</v>
       </c>
-      <c r="V8" s="87">
+      <c r="V8" s="104">
         <v>17</v>
       </c>
-      <c r="W8" s="87">
+      <c r="W8" s="104">
         <v>18</v>
       </c>
-      <c r="X8" s="87">
+      <c r="X8" s="104">
         <v>19</v>
       </c>
-      <c r="Y8" s="87">
+      <c r="Y8" s="104">
         <v>20</v>
       </c>
-      <c r="Z8" s="87">
+      <c r="Z8" s="104">
         <v>21</v>
       </c>
-      <c r="AA8" s="87">
+      <c r="AA8" s="104">
         <v>22</v>
       </c>
-      <c r="AB8" s="87">
+      <c r="AB8" s="104">
         <v>23</v>
       </c>
-      <c r="AC8" s="87">
+      <c r="AC8" s="104">
         <v>24</v>
       </c>
-      <c r="AD8" s="87">
+      <c r="AD8" s="104">
         <v>25</v>
       </c>
-      <c r="AE8" s="87">
+      <c r="AE8" s="104">
         <v>26</v>
       </c>
-      <c r="AF8" s="87">
+      <c r="AF8" s="104">
         <v>27</v>
       </c>
-      <c r="AG8" s="87">
+      <c r="AG8" s="104">
         <v>28</v>
       </c>
-      <c r="AH8" s="87">
+      <c r="AH8" s="104">
         <v>29</v>
       </c>
-      <c r="AI8" s="87">
+      <c r="AI8" s="104">
         <v>30</v>
       </c>
-      <c r="AJ8" s="103">
+      <c r="AJ8" s="106">
         <v>31</v>
       </c>
-      <c r="AK8" s="105" t="s">
+      <c r="AK8" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="AL8" s="107" t="s">
+      <c r="AL8" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="AM8" s="100" t="s">
+      <c r="AM8" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="AN8" s="95" t="s">
+      <c r="AN8" s="123" t="s">
         <v>11</v>
       </c>
-      <c r="AO8" s="96"/>
-      <c r="AP8" s="95" t="s">
+      <c r="AO8" s="124"/>
+      <c r="AP8" s="123" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="97"/>
+      <c r="AQ8" s="125"/>
     </row>
     <row r="9" spans="1:44" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="77"/>
-      <c r="B9" s="74"/>
-      <c r="C9" s="77"/>
-      <c r="D9" s="80"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="99"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="88"/>
-      <c r="L9" s="88"/>
-      <c r="M9" s="88"/>
-      <c r="N9" s="88"/>
-      <c r="O9" s="88"/>
-      <c r="P9" s="88"/>
-      <c r="Q9" s="88"/>
-      <c r="R9" s="88"/>
-      <c r="S9" s="88"/>
-      <c r="T9" s="88"/>
-      <c r="U9" s="88"/>
-      <c r="V9" s="88"/>
-      <c r="W9" s="88"/>
-      <c r="X9" s="88"/>
-      <c r="Y9" s="88"/>
-      <c r="Z9" s="88"/>
-      <c r="AA9" s="88"/>
-      <c r="AB9" s="88"/>
-      <c r="AC9" s="88"/>
-      <c r="AD9" s="88"/>
-      <c r="AE9" s="88"/>
-      <c r="AF9" s="88"/>
-      <c r="AG9" s="88"/>
-      <c r="AH9" s="88"/>
-      <c r="AI9" s="88"/>
-      <c r="AJ9" s="104"/>
-      <c r="AK9" s="106"/>
-      <c r="AL9" s="108"/>
-      <c r="AM9" s="101"/>
+      <c r="A9" s="116"/>
+      <c r="B9" s="130"/>
+      <c r="C9" s="116"/>
+      <c r="D9" s="133"/>
+      <c r="E9" s="136"/>
+      <c r="F9" s="127"/>
+      <c r="G9" s="105"/>
+      <c r="H9" s="105"/>
+      <c r="I9" s="105"/>
+      <c r="J9" s="105"/>
+      <c r="K9" s="105"/>
+      <c r="L9" s="105"/>
+      <c r="M9" s="105"/>
+      <c r="N9" s="105"/>
+      <c r="O9" s="105"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
+      <c r="R9" s="105"/>
+      <c r="S9" s="105"/>
+      <c r="T9" s="105"/>
+      <c r="U9" s="105"/>
+      <c r="V9" s="105"/>
+      <c r="W9" s="105"/>
+      <c r="X9" s="105"/>
+      <c r="Y9" s="105"/>
+      <c r="Z9" s="105"/>
+      <c r="AA9" s="105"/>
+      <c r="AB9" s="105"/>
+      <c r="AC9" s="105"/>
+      <c r="AD9" s="105"/>
+      <c r="AE9" s="105"/>
+      <c r="AF9" s="105"/>
+      <c r="AG9" s="105"/>
+      <c r="AH9" s="105"/>
+      <c r="AI9" s="105"/>
+      <c r="AJ9" s="107"/>
+      <c r="AK9" s="109"/>
+      <c r="AL9" s="111"/>
+      <c r="AM9" s="102"/>
       <c r="AN9" s="4" t="s">
         <v>12</v>
       </c>
@@ -7496,6 +7496,34 @@
     </row>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:AJ7"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="AE8:AE9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="AN8:AO8"/>
+    <mergeCell ref="AP8:AQ8"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S9"/>
     <mergeCell ref="AM8:AM9"/>
     <mergeCell ref="A3:AQ3"/>
     <mergeCell ref="AF8:AF9"/>
@@ -7512,34 +7540,6 @@
     <mergeCell ref="AL8:AL9"/>
     <mergeCell ref="AK7:AQ7"/>
     <mergeCell ref="A7:A9"/>
-    <mergeCell ref="AN8:AO8"/>
-    <mergeCell ref="AP8:AQ8"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:AJ7"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="AE8:AE9"/>
-    <mergeCell ref="T8:T9"/>
   </mergeCells>
   <pageMargins left="0.27559055118110237" right="0.23622047244094491" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="77" orientation="landscape" r:id="rId1"/>
@@ -7576,51 +7576,51 @@
       <c r="AO1" s="2"/>
     </row>
     <row r="3" spans="1:44" ht="29.25" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="102"/>
-      <c r="S3" s="102"/>
-      <c r="T3" s="102"/>
-      <c r="U3" s="102"/>
-      <c r="V3" s="102"/>
-      <c r="W3" s="102"/>
-      <c r="X3" s="102"/>
-      <c r="Y3" s="102"/>
-      <c r="Z3" s="102"/>
-      <c r="AA3" s="102"/>
-      <c r="AB3" s="102"/>
-      <c r="AC3" s="102"/>
-      <c r="AD3" s="102"/>
-      <c r="AE3" s="102"/>
-      <c r="AF3" s="102"/>
-      <c r="AG3" s="102"/>
-      <c r="AH3" s="102"/>
-      <c r="AI3" s="102"/>
-      <c r="AJ3" s="102"/>
-      <c r="AK3" s="102"/>
-      <c r="AL3" s="102"/>
-      <c r="AM3" s="102"/>
-      <c r="AN3" s="102"/>
-      <c r="AO3" s="102"/>
-      <c r="AP3" s="102"/>
-      <c r="AQ3" s="102"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="103"/>
+      <c r="Q3" s="103"/>
+      <c r="R3" s="103"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="103"/>
+      <c r="X3" s="103"/>
+      <c r="Y3" s="103"/>
+      <c r="Z3" s="103"/>
+      <c r="AA3" s="103"/>
+      <c r="AB3" s="103"/>
+      <c r="AC3" s="103"/>
+      <c r="AD3" s="103"/>
+      <c r="AE3" s="103"/>
+      <c r="AF3" s="103"/>
+      <c r="AG3" s="103"/>
+      <c r="AH3" s="103"/>
+      <c r="AI3" s="103"/>
+      <c r="AJ3" s="103"/>
+      <c r="AK3" s="103"/>
+      <c r="AL3" s="103"/>
+      <c r="AM3" s="103"/>
+      <c r="AN3" s="103"/>
+      <c r="AO3" s="103"/>
+      <c r="AP3" s="103"/>
+      <c r="AQ3" s="103"/>
     </row>
     <row r="4" spans="1:44" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F4" s="2" t="s">
@@ -7746,221 +7746,221 @@
       <c r="AQ6" s="32"/>
     </row>
     <row r="7" spans="1:44" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="140" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="143" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="130" t="s">
+      <c r="C7" s="140" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="136" t="s">
+      <c r="D7" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="139" t="s">
+      <c r="E7" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="142" t="s">
+      <c r="F7" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="143"/>
-      <c r="H7" s="143"/>
-      <c r="I7" s="143"/>
-      <c r="J7" s="143"/>
-      <c r="K7" s="143"/>
-      <c r="L7" s="143"/>
-      <c r="M7" s="143"/>
-      <c r="N7" s="143"/>
-      <c r="O7" s="143"/>
-      <c r="P7" s="143"/>
-      <c r="Q7" s="143"/>
-      <c r="R7" s="143"/>
-      <c r="S7" s="143"/>
-      <c r="T7" s="143"/>
-      <c r="U7" s="143"/>
-      <c r="V7" s="143"/>
-      <c r="W7" s="143"/>
-      <c r="X7" s="143"/>
-      <c r="Y7" s="143"/>
-      <c r="Z7" s="143"/>
-      <c r="AA7" s="143"/>
-      <c r="AB7" s="143"/>
-      <c r="AC7" s="143"/>
-      <c r="AD7" s="143"/>
-      <c r="AE7" s="143"/>
-      <c r="AF7" s="143"/>
-      <c r="AG7" s="143"/>
-      <c r="AH7" s="143"/>
-      <c r="AI7" s="143"/>
-      <c r="AJ7" s="144"/>
-      <c r="AK7" s="145" t="s">
+      <c r="G7" s="153"/>
+      <c r="H7" s="153"/>
+      <c r="I7" s="153"/>
+      <c r="J7" s="153"/>
+      <c r="K7" s="153"/>
+      <c r="L7" s="153"/>
+      <c r="M7" s="153"/>
+      <c r="N7" s="153"/>
+      <c r="O7" s="153"/>
+      <c r="P7" s="153"/>
+      <c r="Q7" s="153"/>
+      <c r="R7" s="153"/>
+      <c r="S7" s="153"/>
+      <c r="T7" s="153"/>
+      <c r="U7" s="153"/>
+      <c r="V7" s="153"/>
+      <c r="W7" s="153"/>
+      <c r="X7" s="153"/>
+      <c r="Y7" s="153"/>
+      <c r="Z7" s="153"/>
+      <c r="AA7" s="153"/>
+      <c r="AB7" s="153"/>
+      <c r="AC7" s="153"/>
+      <c r="AD7" s="153"/>
+      <c r="AE7" s="153"/>
+      <c r="AF7" s="153"/>
+      <c r="AG7" s="153"/>
+      <c r="AH7" s="153"/>
+      <c r="AI7" s="153"/>
+      <c r="AJ7" s="154"/>
+      <c r="AK7" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="AL7" s="145"/>
-      <c r="AM7" s="145"/>
-      <c r="AN7" s="145"/>
-      <c r="AO7" s="145"/>
-      <c r="AP7" s="145"/>
-      <c r="AQ7" s="146"/>
+      <c r="AL7" s="155"/>
+      <c r="AM7" s="155"/>
+      <c r="AN7" s="155"/>
+      <c r="AO7" s="155"/>
+      <c r="AP7" s="155"/>
+      <c r="AQ7" s="156"/>
     </row>
     <row r="8" spans="1:44" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="131"/>
-      <c r="B8" s="134"/>
-      <c r="C8" s="131"/>
-      <c r="D8" s="137"/>
-      <c r="E8" s="140"/>
-      <c r="F8" s="147">
+      <c r="A8" s="141"/>
+      <c r="B8" s="144"/>
+      <c r="C8" s="141"/>
+      <c r="D8" s="147"/>
+      <c r="E8" s="150"/>
+      <c r="F8" s="157">
         <v>1</v>
       </c>
-      <c r="G8" s="114">
+      <c r="G8" s="159">
         <v>2</v>
       </c>
-      <c r="H8" s="114">
+      <c r="H8" s="159">
         <v>3</v>
       </c>
-      <c r="I8" s="114">
+      <c r="I8" s="159">
         <v>4</v>
       </c>
-      <c r="J8" s="114">
+      <c r="J8" s="159">
         <v>5</v>
       </c>
-      <c r="K8" s="114">
+      <c r="K8" s="159">
         <v>6</v>
       </c>
-      <c r="L8" s="114">
+      <c r="L8" s="159">
         <v>7</v>
       </c>
-      <c r="M8" s="114">
+      <c r="M8" s="159">
         <v>8</v>
       </c>
-      <c r="N8" s="114">
+      <c r="N8" s="159">
         <v>9</v>
       </c>
-      <c r="O8" s="114">
+      <c r="O8" s="159">
         <v>10</v>
       </c>
-      <c r="P8" s="114">
+      <c r="P8" s="159">
         <v>11</v>
       </c>
-      <c r="Q8" s="114">
+      <c r="Q8" s="159">
         <v>12</v>
       </c>
-      <c r="R8" s="114">
+      <c r="R8" s="159">
         <v>13</v>
       </c>
-      <c r="S8" s="114">
+      <c r="S8" s="159">
         <v>14</v>
       </c>
-      <c r="T8" s="114">
+      <c r="T8" s="159">
         <v>15</v>
       </c>
-      <c r="U8" s="114">
+      <c r="U8" s="159">
         <v>16</v>
       </c>
-      <c r="V8" s="114">
+      <c r="V8" s="159">
         <v>17</v>
       </c>
-      <c r="W8" s="114">
+      <c r="W8" s="159">
         <v>18</v>
       </c>
-      <c r="X8" s="114">
+      <c r="X8" s="159">
         <v>19</v>
       </c>
-      <c r="Y8" s="114">
+      <c r="Y8" s="159">
         <v>20</v>
       </c>
-      <c r="Z8" s="114">
+      <c r="Z8" s="159">
         <v>21</v>
       </c>
-      <c r="AA8" s="114">
+      <c r="AA8" s="159">
         <v>22</v>
       </c>
-      <c r="AB8" s="114">
+      <c r="AB8" s="159">
         <v>23</v>
       </c>
-      <c r="AC8" s="114">
+      <c r="AC8" s="159">
         <v>24</v>
       </c>
-      <c r="AD8" s="114">
+      <c r="AD8" s="159">
         <v>25</v>
       </c>
-      <c r="AE8" s="114">
+      <c r="AE8" s="159">
         <v>26</v>
       </c>
-      <c r="AF8" s="114">
+      <c r="AF8" s="159">
         <v>27</v>
       </c>
-      <c r="AG8" s="114">
+      <c r="AG8" s="159">
         <v>28</v>
       </c>
-      <c r="AH8" s="114">
+      <c r="AH8" s="159">
         <v>29</v>
       </c>
-      <c r="AI8" s="114">
+      <c r="AI8" s="159">
         <v>30</v>
       </c>
-      <c r="AJ8" s="116">
+      <c r="AJ8" s="164">
         <v>31</v>
       </c>
-      <c r="AK8" s="118" t="s">
+      <c r="AK8" s="166" t="s">
         <v>14</v>
       </c>
-      <c r="AL8" s="120" t="s">
+      <c r="AL8" s="168" t="s">
         <v>13</v>
       </c>
-      <c r="AM8" s="122" t="s">
+      <c r="AM8" s="170" t="s">
         <v>9</v>
       </c>
-      <c r="AN8" s="124" t="s">
+      <c r="AN8" s="172" t="s">
         <v>11</v>
       </c>
-      <c r="AO8" s="125"/>
-      <c r="AP8" s="124" t="s">
+      <c r="AO8" s="173"/>
+      <c r="AP8" s="172" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="126"/>
+      <c r="AQ8" s="174"/>
     </row>
     <row r="9" spans="1:44" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="132"/>
-      <c r="B9" s="135"/>
-      <c r="C9" s="132"/>
-      <c r="D9" s="138"/>
-      <c r="E9" s="141"/>
-      <c r="F9" s="148"/>
-      <c r="G9" s="115"/>
-      <c r="H9" s="115"/>
-      <c r="I9" s="115"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="115"/>
-      <c r="L9" s="115"/>
-      <c r="M9" s="115"/>
-      <c r="N9" s="115"/>
-      <c r="O9" s="115"/>
-      <c r="P9" s="115"/>
-      <c r="Q9" s="115"/>
-      <c r="R9" s="115"/>
-      <c r="S9" s="115"/>
-      <c r="T9" s="115"/>
-      <c r="U9" s="115"/>
-      <c r="V9" s="115"/>
-      <c r="W9" s="115"/>
-      <c r="X9" s="115"/>
-      <c r="Y9" s="115"/>
-      <c r="Z9" s="115"/>
-      <c r="AA9" s="115"/>
-      <c r="AB9" s="115"/>
-      <c r="AC9" s="115"/>
-      <c r="AD9" s="115"/>
-      <c r="AE9" s="115"/>
-      <c r="AF9" s="115"/>
-      <c r="AG9" s="115"/>
-      <c r="AH9" s="115"/>
-      <c r="AI9" s="115"/>
-      <c r="AJ9" s="117"/>
-      <c r="AK9" s="119"/>
-      <c r="AL9" s="121"/>
-      <c r="AM9" s="123"/>
+      <c r="A9" s="142"/>
+      <c r="B9" s="145"/>
+      <c r="C9" s="142"/>
+      <c r="D9" s="148"/>
+      <c r="E9" s="151"/>
+      <c r="F9" s="158"/>
+      <c r="G9" s="160"/>
+      <c r="H9" s="160"/>
+      <c r="I9" s="160"/>
+      <c r="J9" s="160"/>
+      <c r="K9" s="160"/>
+      <c r="L9" s="160"/>
+      <c r="M9" s="160"/>
+      <c r="N9" s="160"/>
+      <c r="O9" s="160"/>
+      <c r="P9" s="160"/>
+      <c r="Q9" s="160"/>
+      <c r="R9" s="160"/>
+      <c r="S9" s="160"/>
+      <c r="T9" s="160"/>
+      <c r="U9" s="160"/>
+      <c r="V9" s="160"/>
+      <c r="W9" s="160"/>
+      <c r="X9" s="160"/>
+      <c r="Y9" s="160"/>
+      <c r="Z9" s="160"/>
+      <c r="AA9" s="160"/>
+      <c r="AB9" s="160"/>
+      <c r="AC9" s="160"/>
+      <c r="AD9" s="160"/>
+      <c r="AE9" s="160"/>
+      <c r="AF9" s="160"/>
+      <c r="AG9" s="160"/>
+      <c r="AH9" s="160"/>
+      <c r="AI9" s="160"/>
+      <c r="AJ9" s="165"/>
+      <c r="AK9" s="167"/>
+      <c r="AL9" s="169"/>
+      <c r="AM9" s="171"/>
       <c r="AN9" s="47" t="s">
         <v>12</v>
       </c>
@@ -8779,15 +8779,15 @@
       <c r="AH27" s="66"/>
       <c r="AI27" s="66"/>
       <c r="AJ27" s="70"/>
-      <c r="AK27" s="127" t="s">
+      <c r="AK27" s="175" t="s">
         <v>10</v>
       </c>
-      <c r="AL27" s="128"/>
-      <c r="AM27" s="128"/>
-      <c r="AN27" s="128"/>
-      <c r="AO27" s="128"/>
-      <c r="AP27" s="128"/>
-      <c r="AQ27" s="129"/>
+      <c r="AL27" s="176"/>
+      <c r="AM27" s="176"/>
+      <c r="AN27" s="176"/>
+      <c r="AO27" s="176"/>
+      <c r="AP27" s="176"/>
+      <c r="AQ27" s="177"/>
     </row>
     <row r="28" spans="1:43" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="67"/>
@@ -8830,15 +8830,15 @@
       <c r="AH28" s="68"/>
       <c r="AI28" s="68"/>
       <c r="AJ28" s="71"/>
-      <c r="AK28" s="111" t="s">
+      <c r="AK28" s="161" t="s">
         <v>6</v>
       </c>
-      <c r="AL28" s="112"/>
-      <c r="AM28" s="112"/>
-      <c r="AN28" s="112"/>
-      <c r="AO28" s="112"/>
-      <c r="AP28" s="112"/>
-      <c r="AQ28" s="113"/>
+      <c r="AL28" s="162"/>
+      <c r="AM28" s="162"/>
+      <c r="AN28" s="162"/>
+      <c r="AO28" s="162"/>
+      <c r="AP28" s="162"/>
+      <c r="AQ28" s="163"/>
     </row>
     <row r="29" spans="1:43" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F29" s="15"/>
@@ -8916,6 +8916,36 @@
     </row>
   </sheetData>
   <mergeCells count="46">
+    <mergeCell ref="AK28:AQ28"/>
+    <mergeCell ref="AF8:AF9"/>
+    <mergeCell ref="AG8:AG9"/>
+    <mergeCell ref="AH8:AH9"/>
+    <mergeCell ref="AI8:AI9"/>
+    <mergeCell ref="AJ8:AJ9"/>
+    <mergeCell ref="AK8:AK9"/>
+    <mergeCell ref="AL8:AL9"/>
+    <mergeCell ref="AM8:AM9"/>
+    <mergeCell ref="AN8:AO8"/>
+    <mergeCell ref="AP8:AQ8"/>
+    <mergeCell ref="AK27:AQ27"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="AE8:AE9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
     <mergeCell ref="A3:AQ3"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="B7:B9"/>
@@ -8932,36 +8962,6 @@
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="AE8:AE9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="AK28:AQ28"/>
-    <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="AG8:AG9"/>
-    <mergeCell ref="AH8:AH9"/>
-    <mergeCell ref="AI8:AI9"/>
-    <mergeCell ref="AJ8:AJ9"/>
-    <mergeCell ref="AK8:AK9"/>
-    <mergeCell ref="AL8:AL9"/>
-    <mergeCell ref="AM8:AM9"/>
-    <mergeCell ref="AN8:AO8"/>
-    <mergeCell ref="AP8:AQ8"/>
-    <mergeCell ref="AK27:AQ27"/>
   </mergeCells>
   <pageMargins left="0.27559055118110237" right="0.23622047244094491" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="79" orientation="landscape" r:id="rId1"/>

</xml_diff>